<commit_message>
Guia Sales v2: nomes reais dos servicos SAP (sessao 22/07) + aba Servicios SAP
Achados decisivos do doc 'Integraciones para cotizar y crear un pedido':
- Z301 = OFERTA/RESERVA e Z300 = PEDIDO DE VENTA (resolve o conflito da
  HU-119 bloco 1c com fonte documental do proprio time SAP)
- Pedido de veiculos e cadeia de 3 passos: ASIG_CLIENTE + MONEDA_CLIENTE
  (prerrequisitos) -> SSA_CREA_ORD_VEH (Z301) -> SSA_COPIA_ORD_VEH (Z300)
- SSA_MOD_ORD_VEH confirmado como rota de modificacao/liberacao (RN-21)
- Consulta materiales tem variante MASIVA (ZHYB_C4C_CONSULTA_MATERIALES)
- Catalogo replica por IDoc MATMAS; retorno por COD_REPLICATE_SALES_ORDER01
  e SalesOrderConfirmationMessage; YMKT_SALES_ORDER inclui RETURNS
- Descuento de vendedor: scheduler vs por pedido segue aberto no doc deles

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ouMFEvRtMPEA2sZAxeatj
</commit_message>
<xml_diff>
--- a/docs/mapeo/Mapeo_de_Datos_SALES.xlsx
+++ b/docs/mapeo/Mapeo_de_Datos_SALES.xlsx
@@ -6,7 +6,8 @@
     <sheet name="Mapeo Campos" sheetId="2" r:id="rId2"/>
     <sheet name="Deduplicacion" sheetId="3" r:id="rId3"/>
     <sheet name="Reglas" sheetId="4" r:id="rId4"/>
-    <sheet name="Fuentes" sheetId="5" r:id="rId5"/>
+    <sheet name="Servicios SAP" sheetId="5" r:id="rId5"/>
+    <sheet name="Fuentes" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -108,7 +109,7 @@
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GUIA SALES - Integraciones Salesforce &lt;-&gt; SAP via MuleSoft (12/08/2026) - 21 interfaces UNICAS, sin duplicados, encajadas en el flujo construido</t>
+          <t xml:space="preserve">GUIA SALES v2 - Integraciones Salesforce &lt;-&gt; SAP via MuleSoft (12/08/2026) - 21 interfaces UNICAS, con los nombres de servicio SAP confirmados en la sesion 22/07</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -386,7 +387,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vehicle Specifications (STAR BOD) / maestro de modelos DBM</t>
+          <t xml:space="preserve">Réplica estándar de materiales SAP: IDoc MATMAS (MATMAS_CFS_MATMAS05) + maestro de modelos DBM</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -448,7 +449,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONSULTA/réplica de maestro de materiales (MARA + MVKE por sociedad/canal)</t>
+          <t xml:space="preserve">Réplica estándar de materiales SAP: IDoc MATMAS (MATMAS_CFS_MATMAS05) — MARA + MVKE por sociedad/canal</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -696,7 +697,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">CONSULTA_MATERIALES (modo masivo) + ZHYB_DBM_TEXTO_EXISTENCIA_RFC</t>
+          <t xml:space="preserve">ZHYB_C4C_CONSULTA_MATERIALES (variante MASIVA — hay request-masivo/response-masivo) + ZHYB_DBM_TEXTO_EXISTENCIA_RFC. Vehículos: ZQEV_C4C_CONSULTA_MATERIALES / ZQEV_SD_CONSULTA_GENERAL_MAT</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1006,7 +1007,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pedido de venta Z301 (bloquea stock) · variantes: N pedidos por VIN en flotas y consolidación al cierre</t>
+          <t xml:space="preserve">VEHÍCULOS (cadena de 3 pasos): ZQEV_ASIG_CLIENTE y ZQEV_MONEDA_CLIENTE (prerrequisitos) → ZQEV_SSA_CREA_ORD_VEH crea la Z301 (OFERTA/RESERVA) → ZQEV_SSA_COPIA_ORD_VEH copia la Z301 a Z300 (PEDIDO DE VENTA). Modificar: ZQEV_SSA_MOD_ORD_VEH (Z301 y Z300). REPUESTOS/PA: ZHYB_MONEDA_CLIENTE + ZHYB_SD_PARAM_CLIENTE → ZHYB_DBM_COTIZA_REP_RFC; PA usa cod_salesorder_simulate (síncrono) + IDoc SALESORDER_CREATEFROMDAT2</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1026,7 +1027,7 @@
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Es el corazón del flujo ya construido: cotización → aceptación → pedido → SAP. La idempotencia es DOBLE (lock en SF + clave en Mule)</t>
+          <t xml:space="preserve">Corazón del flujo construido (cotización → aceptación → pedido → SAP). Idempotencia DOBLE (lock FOR UPDATE en SF + clave en Mule). PEDIDO PARA MULE: exponer UNA Experience API que orqueste internamente prerrequisitos + CREA + COPIA; Salesforce no debe encadenar 3-4 llamadas</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
@@ -1068,7 +1069,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Confirmación de pedido / factura (IDoc de retorno)</t>
+          <t xml:space="preserve">COD_REPLICATE_SALES_ORDER01 (réplica de la orden creada) · SalesOrderConfirmationMessage / COD_SALESORDER_CONFIRMATION (confirma y cierra) · YMKT_SALES_ORDER (Quotations/Orders/Returns replication)</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1192,7 +1193,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z301 (fecha de vigencia como parámetro) · ZQEV_SSA_MOD_ORD_VEH / ZQEV_DBM_RECHAZAR_RESERVA (a confirmar por el equipo SAP)</t>
+          <t xml:space="preserve">ZQEV_SSA_MOD_ORD_VEH — CONFIRMADO en la sesión 22/07 que modifica Z301 (reserva) y Z300 (pedido): es la ruta de la liberación anticipada. ZQEV_DBM_RECHAZAR_RESERVA para el rechazo</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1254,7 +1255,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Documento de devolución por dominio: peças Z111 (confirmado); vehículos y PA A CONFIRMAR por el equipo SAP</t>
+          <t xml:space="preserve">Peças: Z111 (confirmado). PA: el canal YMKT_SALES_ORDER ya replica Quotations/Orders/RETURNS — pista a validar con el equipo SAP. Vehículos: A CONFIRMAR</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -3222,6 +3223,695 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="16" customWidth="1"/>
+    <col min="2" max="2" width="46" customWidth="1"/>
+    <col min="3" max="3" width="56" customWidth="1"/>
+    <col min="4" max="4" width="20" customWidth="1"/>
+    <col min="5" max="5" width="60" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catalogo de servicios SAP confirmados en la sesion 22/07 (documento Integraciones para cotizar y crear un pedido)</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="E2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dominio</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Servicio / función SAP</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Para qué sirve (según la sesión 22/07)</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interfaz de esta guía</t>
+        </is>
+      </c>
+      <c r="E3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_ASIG_CLIENTE</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prerrequisito obligatorio antes de ejecutar cualquier función de pedido</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Debe ir DENTRO de la orquestación Mule, no como llamada separada desde Salesforce</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_MONEDA_CLIENTE</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Prerrequisito obligatorio (moneda del cliente)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ídem</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_SSA_CREA_ORD_VEH</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crea la Z301 = OFERTA o RESERVA</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12 / INT-SAL-15</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Aquí se bloquea el stock: es la reserva</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_SSA_COPIA_ORD_VEH</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Toma la Z301 y la copia a Z300 = PEDIDO DE VENTA</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El pedido NO es una sola llamada: es crear y luego copiar</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_SSA_MOD_ORD_VEH</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modifica Z301 (reserva) y Z300 (pedido)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-14 / INT-SAL-15</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ruta de la liberación anticipada y de la modificación</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vehículos</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZQEV_C4C_CONSULTA_MATERIALES / ZQEV_SD_CONSULTA_GENERAL_MAT</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consulta de materiales del lado vehículos</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-07</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_C4C_CONSULTA_MATERIALES</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consulta de materiales para agregar a la orden: uno a uno o CARGA MASIVA</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-07</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">USAR LA VARIANTE MASIVA: una llamada por lote (ya es lo que hace el grid)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">TDET_SALDOS = PISO − RESERVA</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cálculo del saldo disponible</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-07</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PUEDE SER NEGATIVO y se devuelve tal cual (no truncar)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_DBM_TEXTO_EXISTENCIA_RFC</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Texto de existencia (ubicación de la pieza)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-07</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">De este texto derivamos Otro Centro / Otra Sociedad</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_MONEDA_CLIENTE + ZHYB_SD_PARAM_CLIENTE</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parámetros y moneda del cliente antes de generar el pedido</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Equivalente de los prerrequisitos de vehículos, para repuestos/PA</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_DBM_COTIZA_REP_RFC</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Crea cotización / pedido de repuestos en el DBM</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_DBM_MOD_DET_ORDEN</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Modifica detalle de la orden/cotización</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-14</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_DBMPOSICIONES</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Consulta de posiciones del pedido</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-14</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">OJO: la guía de historias la nombra ZQEV_DBMPOSICIONES y la sesión 22/07 ZHYB_DBMPOSICIONES — confirmar el nombre exacto con el equipo SAP</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Repuestos</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_DBM_DESCUENTO_DE_VENDEDOR</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tope de descuento del vendedor</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DECISIÓN ABIERTA en el propio documento: scheduler diario en lugar de consultar en cada pedido. Recomendación: scheduler + caché (evita una llamada por cotización)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">cod_salesorder_simulate</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Simulación de precio del pedido — SÍNCRONO</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El precio lo calcula el SD: Salesforce exhibe y congela</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SALESORDER_CREATEFROMDAT2 (IDoc)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirma / crea el pedido en SD</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El resto del flujo de PA es asíncrono por IDocs</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COD_REPLICATE_SALES_ORDER01</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Respuesta con la orden creada</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-13</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Es el retorno que alimenta SapOrderResponse__e</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">COD_SALESORDER_CONFIRMATION / SalesOrderConfirmationMessage</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Confirma y cierra la orden</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-13</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PA</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YMKT_SALES_ORDER</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Replicación de Quotations / Orders / RETURNS</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-13 / INT-SAL-16</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contiene RETURNS: posible ruta de devoluciones para PA — validar</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Catálogo</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MATMAS (MATMAS_CFS_MATMAS05)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Réplica estándar de materiales de SAP</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-02 / INT-SAL-03</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Es el contrato de la réplica de catálogo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clientes</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ZHYB_SD_PARAM_CLIENTE / Update Business Partner</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parámetros del cliente y actualización de BP</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-10</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B2C (fuera de Sales)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Archivos XML en SFTP + scheduler Mule</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Estrategia B2C: B2C genera XML en SFTP y Mule los lee</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">No aplica a Sales</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ATENCIÓN: el documento circula con credenciales SFTP en texto plano — deben rotarse y salir del documento</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="46" customWidth="1"/>
     <col min="2" max="2" width="80" customWidth="1"/>
   </cols>
@@ -3373,10 +4063,22 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">Catálogo de servicios de cotización y pedido (Z300/Z301, prerrequisitos, IDocs)</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documento del equipo SAP/Mule "Integraciones para cotizar y crear un pedido" — sesión 22/07/2026 (fuente primaria de los nombres de función)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">Premisa STAR 5 (BODs de cliente, catálogo e inventario)</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">Documento del equipo (inspección de 870 XSDs) — premisa del programa, a confirmar en el contrato Mule</t>
         </is>

</xml_diff>

<commit_message>
Guia Sales v3: coluna com o item de estimativa MuleSoft + aba de visao inversa
- Coluna 'Item de estimacion MuleSoft (vista S4)' em cada uma das 21
  interfaces (Pedidos Outbound / Inventario 03-01B-C-D / Captura Leads /
  Documentacion), marcando as que nao aparecem na vista compartilhada
- Nova aba 'Estimacion Mule': por item, quais interfaces cobre + 3 lacunas
  de cobertura (catalogo+precos, disponibilidade+criacao de material,
  clientes) e as duvidas do item 'Outbound' (retorno e modificacao inbound)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012ouMFEvRtMPEA2sZAxeatj
</commit_message>
<xml_diff>
--- a/docs/mapeo/Mapeo_de_Datos_SALES.xlsx
+++ b/docs/mapeo/Mapeo_de_Datos_SALES.xlsx
@@ -6,8 +6,9 @@
     <sheet name="Mapeo Campos" sheetId="2" r:id="rId2"/>
     <sheet name="Deduplicacion" sheetId="3" r:id="rId3"/>
     <sheet name="Reglas" sheetId="4" r:id="rId4"/>
-    <sheet name="Servicios SAP" sheetId="5" r:id="rId5"/>
-    <sheet name="Fuentes" sheetId="6" r:id="rId6"/>
+    <sheet name="Estimacion Mule" sheetId="5" r:id="rId5"/>
+    <sheet name="Servicios SAP" sheetId="6" r:id="rId6"/>
+    <sheet name="Fuentes" sheetId="7" r:id="rId7"/>
   </sheets>
 </workbook>
 </file>
@@ -104,12 +105,13 @@
     <col min="10" max="10" width="30" customWidth="1"/>
     <col min="11" max="11" width="46" customWidth="1"/>
     <col min="12" max="12" width="34" customWidth="1"/>
+    <col min="13" max="13" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GUIA SALES v2 - Integraciones Salesforce &lt;-&gt; SAP via MuleSoft (12/08/2026) - 21 interfaces UNICAS, con los nombres de servicio SAP confirmados en la sesion 22/07</t>
+          <t xml:space="preserve">GUIA SALES v3 - Integraciones Salesforce &lt;-&gt; SAP via MuleSoft (12/08/2026) - 21 interfaces UNICAS, con nombres de servicio SAP (sesion 22/07) y vinculacion a los items de estimacion MuleSoft (vista S4)</t>
         </is>
       </c>
       <c r="B1" s="3" t="inlineStr">
@@ -163,6 +165,11 @@
         </is>
       </c>
       <c r="L1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve"/>
         </is>
@@ -229,6 +236,11 @@
           <t xml:space="preserve"/>
         </is>
       </c>
+      <c r="M2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -291,6 +303,11 @@
           <t xml:space="preserve">Historias consolidadas</t>
         </is>
       </c>
+      <c r="M3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ítem de estimación MuleSoft (vista S4)</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -353,6 +370,11 @@
           <t xml:space="preserve">US-SAL-01-02A</t>
         </is>
       </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -415,6 +437,11 @@
           <t xml:space="preserve">US-SAL-02-01A</t>
         </is>
       </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -477,6 +504,11 @@
           <t xml:space="preserve">US-SAL-02-01C (parte catálogo)</t>
         </is>
       </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -539,6 +571,11 @@
           <t xml:space="preserve">US-SAL-02-01B</t>
         </is>
       </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -601,6 +638,11 @@
           <t xml:space="preserve">US-SAL-02-01D</t>
         </is>
       </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -663,6 +705,11 @@
           <t xml:space="preserve">US-SAL-03-01A + US-SAL-03-01D (mismo canal, distinta operación — consolidadas)</t>
         </is>
       </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inventario US-SAL-03-01B, US-SAL-03-01C, US-SAL-03-01D (Parte 1 y Parte 2) — cubre US-SAL-03-01D (estado de la unidad). OJO: 03-01A (alta de unidad) no está nombrada en el ítem</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -725,6 +772,11 @@
           <t xml:space="preserve">US-SAL-02-01C (parte stock real-time)</t>
         </is>
       </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (es la consulta que usa el grid de Repuestos: sin ella la HU-043 no funciona)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -787,6 +839,11 @@
           <t xml:space="preserve">US-021 (no estaba en la guía de integraciones)</t>
         </is>
       </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (US-021 — creación de material desde el flujo guiado)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -849,6 +906,11 @@
           <t xml:space="preserve">US-SAL-01-01A + US-SAL-01-01B + US-SAL-01-01C (mismo canal — consolidadas)</t>
         </is>
       </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clientes — pedido como ADICIONAL por el equipo; no está en la vista S4</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -911,6 +973,11 @@
           <t xml:space="preserve">HU-017 (RN-01/RN-05/RN-26) — sin fila propia en la guía original</t>
         </is>
       </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clientes — pedido como ADICIONAL por el equipo; no está en la vista S4</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -973,6 +1040,11 @@
           <t xml:space="preserve">HU-119 RN-26</t>
         </is>
       </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Clientes — pedido como ADICIONAL por el equipo; no está en la vista S4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1035,6 +1107,11 @@
           <t xml:space="preserve">US-SAL-08-01A + US-SAL-08-01B + US-SAL-08-01C (mismo servicio, distinta cardinalidad — consolidadas)</t>
         </is>
       </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedidos SF → SAP (Outbound)</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1097,6 +1174,11 @@
           <t xml:space="preserve">Retorno de US-SAL-08-01A (estaba implícito)</t>
         </is>
       </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedidos SF → SAP (Outbound) — ¿INCLUIDO? El ítem dice "Outbound" y esto es el RETORNO (inbound): confirmar que no quedó fuera</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1159,6 +1241,11 @@
           <t xml:space="preserve">HU-119 RN-06 — sin fila propia en la guía original</t>
         </is>
       </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedidos SF → SAP (Outbound) — ¿INCLUIDO? Modificación en SAP es inbound: confirmar</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1221,6 +1308,11 @@
           <t xml:space="preserve">US-SAL-03-01B + US-SAL-03-01C (la lógica de timer es 100% Salesforce; solo la liberación es interfaz — consolidadas)</t>
         </is>
       </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inventario US-SAL-03-01B, US-SAL-03-01C, US-SAL-03-01D (Parte 1 y Parte 2) — cubre US-SAL-03-01B/C. En Salesforce el timer ya es nuestro; de Mule solo se necesita la liberación</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1283,6 +1375,11 @@
           <t xml:space="preserve">HU-119 RN-22 + PROP-INT-05 (SOLPED, relacionado)</t>
         </is>
       </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (devolución: NO estimar hasta que SAP defina el documento)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1345,6 +1442,11 @@
           <t xml:space="preserve">US-SAL-04-01A + 04-01B + 04-01C + 04-01D + 04-01F (5 filas → 1 interfaz). 04-01E (showroom) NO es integración: es captura nativa</t>
         </is>
       </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Captura Leads (Sales Lead BOD + custom) Parte 1 y Parte 2</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1407,6 +1509,11 @@
           <t xml:space="preserve">US-SAL-05-01A (+ 05-01C caché, + 05-01D fallas: son reglas de la misma interfaz)</t>
         </is>
       </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (LexisNexis — validación de leads, US-SAL-05-01A)</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -1469,6 +1576,11 @@
           <t xml:space="preserve">US-SAL-05-01B (+ 05-01C/D)</t>
         </is>
       </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (buró EFX — verificar solapamiento con E-CQ de Digital Lending para no pagar dos consultas)</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1531,6 +1643,11 @@
           <t xml:space="preserve">US-SAL-13-01A + US-SAL-13-01B (consolidadas). 13-01C excluida (nativa)</t>
         </is>
       </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentación (OpenText + Document Templates) — la parte OpenText. Document Templates es NATIVO: no consume esfuerzo Mule</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1591,6 +1708,11 @@
       <c r="L24" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">US-SAL-01-02B (una sola interfaz para todas las entidades)</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NO aparece en la vista S4 compartida — confirmar si está estimado en otro sprint (reconciliación mensual)</t>
         </is>
       </c>
     </row>
@@ -3223,6 +3345,283 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
+    <col min="1" max="1" width="46" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="80" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vista inversa: cada item de estimacion MuleSoft (vista S4) y las interfaces que cubre — incluye los huecos de cobertura</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="B2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="C2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="D2" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ítem de estimación MuleSoft</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Equipo</t>
+        </is>
+      </c>
+      <c r="C3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Interfaces de esta guía que cubre</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cobertura / observación</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedidos SF → SAP (Outbound)</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Automotive Sales</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-12 (envío del pedido)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El nombre dice OUTBOUND. El flujo necesita además el RETORNO (INT-SAL-13: número de pedido, confirmación, factura) y la MODIFICACIÓN en SAP (INT-SAL-14). CONFIRMAR si están dentro del ítem o si falta estimarlos. Nota: el pedido de vehículos es una cadena (prerrequisitos → CREA Z301 → COPIA Z300), no una llamada</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Inventario US-SAL-03-01B, US-SAL-03-01C, US-SAL-03-01D (Parte 1 y Parte 2)</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Automotive Sales</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-06 (estado de la unidad) + INT-SAL-15 (liberación de la reserva)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">El ítem nombra 03-01B/C/D. Falta nombrar 03-01A (recepción del inventario unitario por VIN), que es lo que puebla Vehicle/Asset. El timer de reserva (15/45 min) es lógica Salesforce: no consume Mule</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Captura Leads (Sales Lead BOD + custom) Parte 1 y Parte 2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Automotive Sales</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-17 (API única de captura de leads)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cubre los 4 orígenes (LeadsBridge, TalkMe, SFCC/marcas, Cyberfuel SOAP) con UN endpoint de upsert; cada origen es una transformación. La captura en showroom es nativa (sin Mule)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Documentación (OpenText + Document Templates)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Automotive Sales</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-20 (documentos a OpenText)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Solo la parte OpenText es integración. Document Templates de Automotive Cloud EE es generación nativa: no debería consumir esfuerzo Mule</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E-CQ-01 — Validación de Avalúo y Revisión de Vendedor de vehículos Terceros</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Digital Lending</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ninguna de esta guía</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Otro equipo. Se relaciona con la HU-045 (usados/consignación) del lado Sales: coordinar para no duplicar la consulta de avalúo</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">E-CQ-09 — Cotizador / Tasa de Referencia SAP (PRIME, TPROFONI, TBPCR)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">[OSF] SOW002 - Digital Lending</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ninguna de esta guía</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Otro equipo, pero es integración con SAP por el MISMO gateway: reutilizar credencial, monitoreo y política de reintentos</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(sin ítem) Catálogo, precios y tipos de cambio</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-02, 03, 04, 05</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RIESGO: sin catálogo ni listas de precios replicadas, la venta guiada no encuentra material ni precio. Es precondición de los ítems ya estimados</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(sin ítem) Disponibilidad de repuestos y creación de material</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-07, INT-SAL-08</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">RIESGO: son las dos llamadas que el grid de Repuestos (HU-043) y la US-021 ya construidos consumen hoy contra el mock</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">(sin ítem) Clientes</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">INT-SAL-09, 10, 11</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pedido por el equipo como adicional — ya está mapeado en esta guía, pueden empezar</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="46" customWidth="1"/>
     <col min="3" max="3" width="56" customWidth="1"/>
@@ -3909,7 +4308,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <cols>
     <col min="1" max="1" width="46" customWidth="1"/>

</xml_diff>